<commit_message>
Relabel workbook heading, set status to pending student review, tighten bond case study
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/bond_duration_reviewed.xlsx
+++ b/downloads/bond_duration_reviewed.xlsx
@@ -439,7 +439,7 @@
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYNTHETIC TEST FILE - hypothetical data for model testing, not real work</x:t>
+          <x:t xml:space="preserve">Bond Duration Analysis — Synthetic-Data Learning Exercise</x:t>
         </x:is>
       </x:c>
       <x:c r="B1" s="15"/>
@@ -902,7 +902,7 @@
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="15" t="str">
-        <x:v>Scope: synthetic fixed-coupon bond exercise; source inputs are preserved, not verified market quotes.</x:v>
+        <x:v>Scope: synthetic fixed-coupon bond exercise. All inputs are hypothetical, not market quotes.</x:v>
       </x:c>
       <x:c r="B15" s="15"/>
       <x:c r="C15" s="15"/>
@@ -977,7 +977,7 @@
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
       <x:c r="A20" s="15" t="str">
-        <x:v>AI assistance corrected formulas and completed scenarios. Abdullah must review before claiming completion.</x:v>
+        <x:v>AI assisted with formula corrections and scenario completion. Pending student review.</x:v>
       </x:c>
       <x:c r="B20" s="15"/>
       <x:c r="C20" s="15"/>
@@ -1340,7 +1340,7 @@
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="12" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYNTHETIC TEST FILE</x:t>
+          <x:t xml:space="preserve">Bond Duration Analysis — Synthetic-Data Learning Exercise</x:t>
         </x:is>
       </x:c>
       <x:c r="B1" s="7"/>

</xml_diff>